<commit_message>
Remove School Type graph and change bottom 10 to bottom 25
</commit_message>
<xml_diff>
--- a/summary_reports.xlsx
+++ b/summary_reports.xlsx
@@ -463,10 +463,10 @@
         <v>1077</v>
       </c>
       <c r="C2" t="n">
-        <v>180</v>
+        <v>256</v>
       </c>
       <c r="D2" t="n">
-        <v>16.71</v>
+        <v>23.77</v>
       </c>
     </row>
     <row r="3">
@@ -479,10 +479,10 @@
         <v>868</v>
       </c>
       <c r="C3" t="n">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="D3" t="n">
-        <v>21.43</v>
+        <v>22.7</v>
       </c>
     </row>
     <row r="4">
@@ -495,10 +495,10 @@
         <v>429</v>
       </c>
       <c r="C4" t="n">
-        <v>243</v>
+        <v>300</v>
       </c>
       <c r="D4" t="n">
-        <v>56.64</v>
+        <v>69.93000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -511,10 +511,10 @@
         <v>274</v>
       </c>
       <c r="C5" t="n">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="D5" t="n">
-        <v>46.72</v>
+        <v>52.19</v>
       </c>
     </row>
     <row r="6">
@@ -543,10 +543,10 @@
         <v>838</v>
       </c>
       <c r="C7" t="n">
-        <v>98</v>
+        <v>161</v>
       </c>
       <c r="D7" t="n">
-        <v>11.69</v>
+        <v>19.21</v>
       </c>
     </row>
     <row r="8">
@@ -575,10 +575,10 @@
         <v>330</v>
       </c>
       <c r="C9" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D9" t="n">
-        <v>29.7</v>
+        <v>30.61</v>
       </c>
     </row>
     <row r="10">
@@ -591,10 +591,10 @@
         <v>625</v>
       </c>
       <c r="C10" t="n">
-        <v>157</v>
+        <v>211</v>
       </c>
       <c r="D10" t="n">
-        <v>25.12</v>
+        <v>33.76</v>
       </c>
     </row>
     <row r="11">
@@ -639,10 +639,10 @@
         <v>354</v>
       </c>
       <c r="C13" t="n">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="D13" t="n">
-        <v>39.83</v>
+        <v>41.81</v>
       </c>
     </row>
     <row r="14">
@@ -655,10 +655,10 @@
         <v>529</v>
       </c>
       <c r="C14" t="n">
-        <v>220</v>
+        <v>265</v>
       </c>
       <c r="D14" t="n">
-        <v>41.59</v>
+        <v>50.09</v>
       </c>
     </row>
     <row r="15">
@@ -671,10 +671,10 @@
         <v>442</v>
       </c>
       <c r="C15" t="n">
-        <v>132</v>
+        <v>173</v>
       </c>
       <c r="D15" t="n">
-        <v>29.86</v>
+        <v>39.14</v>
       </c>
     </row>
     <row r="16">
@@ -687,10 +687,10 @@
         <v>231</v>
       </c>
       <c r="C16" t="n">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="D16" t="n">
-        <v>53.25</v>
+        <v>59.74</v>
       </c>
     </row>
     <row r="17">
@@ -703,10 +703,10 @@
         <v>528</v>
       </c>
       <c r="C17" t="n">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D17" t="n">
-        <v>37.5</v>
+        <v>37.69</v>
       </c>
     </row>
     <row r="18">
@@ -719,10 +719,10 @@
         <v>324</v>
       </c>
       <c r="C18" t="n">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="D18" t="n">
-        <v>25.62</v>
+        <v>32.41</v>
       </c>
     </row>
     <row r="19">
@@ -735,10 +735,10 @@
         <v>524</v>
       </c>
       <c r="C19" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D19" t="n">
-        <v>30.15</v>
+        <v>30.34</v>
       </c>
     </row>
     <row r="20">
@@ -751,10 +751,10 @@
         <v>290</v>
       </c>
       <c r="C20" t="n">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="D20" t="n">
-        <v>66.20999999999999</v>
+        <v>69.31</v>
       </c>
     </row>
     <row r="21">
@@ -783,10 +783,10 @@
         <v>580</v>
       </c>
       <c r="C22" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D22" t="n">
-        <v>19.31</v>
+        <v>19.48</v>
       </c>
     </row>
     <row r="23">
@@ -799,10 +799,10 @@
         <v>561</v>
       </c>
       <c r="C23" t="n">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D23" t="n">
-        <v>22.82</v>
+        <v>23.35</v>
       </c>
     </row>
     <row r="24">
@@ -847,10 +847,10 @@
         <v>323</v>
       </c>
       <c r="C26" t="n">
-        <v>111</v>
+        <v>157</v>
       </c>
       <c r="D26" t="n">
-        <v>34.37</v>
+        <v>48.61</v>
       </c>
     </row>
     <row r="27">
@@ -863,10 +863,10 @@
         <v>463</v>
       </c>
       <c r="C27" t="n">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="D27" t="n">
-        <v>54.21</v>
+        <v>55.72</v>
       </c>
     </row>
     <row r="28">
@@ -879,10 +879,10 @@
         <v>614</v>
       </c>
       <c r="C28" t="n">
-        <v>243</v>
+        <v>287</v>
       </c>
       <c r="D28" t="n">
-        <v>39.58</v>
+        <v>46.74</v>
       </c>
     </row>
     <row r="29">
@@ -895,10 +895,10 @@
         <v>389</v>
       </c>
       <c r="C29" t="n">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="D29" t="n">
-        <v>39.33</v>
+        <v>41.39</v>
       </c>
     </row>
     <row r="30">
@@ -911,10 +911,10 @@
         <v>455</v>
       </c>
       <c r="C30" t="n">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="D30" t="n">
-        <v>53.41</v>
+        <v>54.73</v>
       </c>
     </row>
     <row r="31">
@@ -943,10 +943,10 @@
         <v>540</v>
       </c>
       <c r="C32" t="n">
-        <v>114</v>
+        <v>154</v>
       </c>
       <c r="D32" t="n">
-        <v>21.11</v>
+        <v>28.52</v>
       </c>
     </row>
     <row r="33">
@@ -959,10 +959,10 @@
         <v>686</v>
       </c>
       <c r="C33" t="n">
-        <v>296</v>
+        <v>318</v>
       </c>
       <c r="D33" t="n">
-        <v>43.15</v>
+        <v>46.36</v>
       </c>
     </row>
     <row r="34">
@@ -991,10 +991,10 @@
         <v>163</v>
       </c>
       <c r="C35" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D35" t="n">
-        <v>74.84999999999999</v>
+        <v>77.3</v>
       </c>
     </row>
     <row r="36">
@@ -1007,10 +1007,10 @@
         <v>631</v>
       </c>
       <c r="C36" t="n">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="D36" t="n">
-        <v>26.47</v>
+        <v>28.53</v>
       </c>
     </row>
     <row r="37">
@@ -1023,10 +1023,10 @@
         <v>385</v>
       </c>
       <c r="C37" t="n">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="D37" t="n">
-        <v>23.12</v>
+        <v>26.49</v>
       </c>
     </row>
     <row r="38">
@@ -1055,10 +1055,10 @@
         <v>828</v>
       </c>
       <c r="C39" t="n">
-        <v>299</v>
+        <v>374</v>
       </c>
       <c r="D39" t="n">
-        <v>36.11</v>
+        <v>45.17</v>
       </c>
     </row>
     <row r="40">
@@ -1071,10 +1071,10 @@
         <v>300</v>
       </c>
       <c r="C40" t="n">
-        <v>191</v>
+        <v>247</v>
       </c>
       <c r="D40" t="n">
-        <v>63.67</v>
+        <v>82.33</v>
       </c>
     </row>
     <row r="41">
@@ -1087,10 +1087,10 @@
         <v>406</v>
       </c>
       <c r="C41" t="n">
-        <v>188</v>
+        <v>206</v>
       </c>
       <c r="D41" t="n">
-        <v>46.31</v>
+        <v>50.74</v>
       </c>
     </row>
     <row r="42">
@@ -1103,10 +1103,10 @@
         <v>385</v>
       </c>
       <c r="C42" t="n">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="D42" t="n">
-        <v>32.73</v>
+        <v>37.66</v>
       </c>
     </row>
     <row r="43">
@@ -1135,10 +1135,10 @@
         <v>873</v>
       </c>
       <c r="C44" t="n">
-        <v>320</v>
+        <v>371</v>
       </c>
       <c r="D44" t="n">
-        <v>36.66</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="45">
@@ -1183,10 +1183,10 @@
         <v>365</v>
       </c>
       <c r="C47" t="n">
-        <v>255</v>
+        <v>279</v>
       </c>
       <c r="D47" t="n">
-        <v>69.86</v>
+        <v>76.44</v>
       </c>
     </row>
     <row r="48">
@@ -1231,10 +1231,10 @@
         <v>1051</v>
       </c>
       <c r="C50" t="n">
-        <v>301</v>
+        <v>329</v>
       </c>
       <c r="D50" t="n">
-        <v>28.64</v>
+        <v>31.3</v>
       </c>
     </row>
     <row r="51">
@@ -1247,10 +1247,10 @@
         <v>320</v>
       </c>
       <c r="C51" t="n">
-        <v>179</v>
+        <v>219</v>
       </c>
       <c r="D51" t="n">
-        <v>55.94</v>
+        <v>68.44</v>
       </c>
     </row>
     <row r="52">
@@ -1263,10 +1263,10 @@
         <v>112</v>
       </c>
       <c r="C52" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D52" t="n">
-        <v>69.64</v>
+        <v>76.79000000000001</v>
       </c>
     </row>
     <row r="53">
@@ -1295,10 +1295,10 @@
         <v>640</v>
       </c>
       <c r="C54" t="n">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="D54" t="n">
-        <v>25</v>
+        <v>26.41</v>
       </c>
     </row>
     <row r="55">
@@ -1311,10 +1311,10 @@
         <v>522</v>
       </c>
       <c r="C55" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="D55" t="n">
-        <v>11.69</v>
+        <v>15.71</v>
       </c>
     </row>
     <row r="56">
@@ -1327,10 +1327,10 @@
         <v>572</v>
       </c>
       <c r="C56" t="n">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="D56" t="n">
-        <v>50</v>
+        <v>52.27</v>
       </c>
     </row>
     <row r="57">
@@ -1343,10 +1343,10 @@
         <v>347</v>
       </c>
       <c r="C57" t="n">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="D57" t="n">
-        <v>41.21</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="58">
@@ -1359,10 +1359,10 @@
         <v>537</v>
       </c>
       <c r="C58" t="n">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="D58" t="n">
-        <v>38.18</v>
+        <v>39.29</v>
       </c>
     </row>
     <row r="59">
@@ -1375,10 +1375,10 @@
         <v>388</v>
       </c>
       <c r="C59" t="n">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="D59" t="n">
-        <v>46.39</v>
+        <v>51.8</v>
       </c>
     </row>
     <row r="60">
@@ -1391,10 +1391,10 @@
         <v>225</v>
       </c>
       <c r="C60" t="n">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="D60" t="n">
-        <v>60.44</v>
+        <v>66.22</v>
       </c>
     </row>
     <row r="61">
@@ -1407,10 +1407,10 @@
         <v>742</v>
       </c>
       <c r="C61" t="n">
-        <v>236</v>
+        <v>254</v>
       </c>
       <c r="D61" t="n">
-        <v>31.81</v>
+        <v>34.23</v>
       </c>
     </row>
     <row r="62">
@@ -1423,10 +1423,10 @@
         <v>1181</v>
       </c>
       <c r="C62" t="n">
-        <v>183</v>
+        <v>206</v>
       </c>
       <c r="D62" t="n">
-        <v>15.5</v>
+        <v>17.44</v>
       </c>
     </row>
     <row r="63">
@@ -1455,10 +1455,10 @@
         <v>266</v>
       </c>
       <c r="C64" t="n">
-        <v>172</v>
+        <v>207</v>
       </c>
       <c r="D64" t="n">
-        <v>64.66</v>
+        <v>77.81999999999999</v>
       </c>
     </row>
     <row r="65">
@@ -1471,10 +1471,10 @@
         <v>452</v>
       </c>
       <c r="C65" t="n">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="D65" t="n">
-        <v>58.63</v>
+        <v>61.5</v>
       </c>
     </row>
     <row r="66">
@@ -1487,10 +1487,10 @@
         <v>262</v>
       </c>
       <c r="C66" t="n">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="D66" t="n">
-        <v>59.54</v>
+        <v>64.89</v>
       </c>
     </row>
     <row r="67">
@@ -1535,10 +1535,10 @@
         <v>150</v>
       </c>
       <c r="C69" t="n">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="D69" t="n">
-        <v>80</v>
+        <v>88.67</v>
       </c>
     </row>
     <row r="70">
@@ -1583,10 +1583,10 @@
         <v>468</v>
       </c>
       <c r="C72" t="n">
-        <v>166</v>
+        <v>315</v>
       </c>
       <c r="D72" t="n">
-        <v>35.47</v>
+        <v>67.31</v>
       </c>
     </row>
     <row r="73">
@@ -1599,10 +1599,10 @@
         <v>239</v>
       </c>
       <c r="C73" t="n">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="D73" t="n">
-        <v>34.31</v>
+        <v>44.35</v>
       </c>
     </row>
     <row r="74">
@@ -1615,10 +1615,10 @@
         <v>395</v>
       </c>
       <c r="C74" t="n">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="D74" t="n">
-        <v>56.2</v>
+        <v>59.24</v>
       </c>
     </row>
     <row r="75">
@@ -1631,10 +1631,10 @@
         <v>435</v>
       </c>
       <c r="C75" t="n">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="D75" t="n">
-        <v>86.90000000000001</v>
+        <v>88.51000000000001</v>
       </c>
     </row>
     <row r="76">
@@ -1647,10 +1647,10 @@
         <v>622</v>
       </c>
       <c r="C76" t="n">
-        <v>228</v>
+        <v>277</v>
       </c>
       <c r="D76" t="n">
-        <v>36.66</v>
+        <v>44.53</v>
       </c>
     </row>
     <row r="77">
@@ -1663,10 +1663,10 @@
         <v>33332</v>
       </c>
       <c r="C77" t="n">
-        <v>11687</v>
+        <v>13091</v>
       </c>
       <c r="D77" t="n">
-        <v>35.06</v>
+        <v>39.27</v>
       </c>
     </row>
   </sheetData>
@@ -1708,161 +1708,161 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UNNAO</t>
+          <t>SHAMLI (PRABUDH NAGAR)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>435</v>
+        <v>150</v>
       </c>
       <c r="C2" t="n">
-        <v>378</v>
+        <v>133</v>
       </c>
       <c r="D2" t="n">
-        <v>86.90000000000001</v>
+        <v>88.67</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SHAMLI (PRABUDH NAGAR)</t>
+          <t>UNNAO</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>150</v>
+        <v>435</v>
       </c>
       <c r="C3" t="n">
-        <v>120</v>
+        <v>385</v>
       </c>
       <c r="D3" t="n">
-        <v>80</v>
+        <v>88.51000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HAPUR (PANCHSHEEL NAGAR)</t>
+          <t>JHANSI</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>163</v>
+        <v>300</v>
       </c>
       <c r="C4" t="n">
-        <v>122</v>
+        <v>247</v>
       </c>
       <c r="D4" t="n">
-        <v>74.84999999999999</v>
+        <v>82.33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>KHERI</t>
+          <t>RAMPUR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>365</v>
+        <v>266</v>
       </c>
       <c r="C5" t="n">
-        <v>255</v>
+        <v>207</v>
       </c>
       <c r="D5" t="n">
-        <v>69.86</v>
+        <v>77.81999999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MAHOBA</t>
+          <t>HAPUR (PANCHSHEEL NAGAR)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>112</v>
+        <v>163</v>
       </c>
       <c r="C6" t="n">
-        <v>78</v>
+        <v>126</v>
       </c>
       <c r="D6" t="n">
-        <v>69.64</v>
+        <v>77.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CHANDAULI</t>
+          <t>MAHOBA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>290</v>
+        <v>112</v>
       </c>
       <c r="C7" t="n">
-        <v>192</v>
+        <v>86</v>
       </c>
       <c r="D7" t="n">
-        <v>66.20999999999999</v>
+        <v>76.79000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SHRAWASTI</t>
+          <t>KHERI</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>130</v>
+        <v>365</v>
       </c>
       <c r="C8" t="n">
-        <v>85</v>
+        <v>279</v>
       </c>
       <c r="D8" t="n">
-        <v>65.38</v>
+        <v>76.44</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RAMPUR</t>
+          <t>AMBEDKAR NAGAR</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>266</v>
+        <v>429</v>
       </c>
       <c r="C9" t="n">
-        <v>172</v>
+        <v>300</v>
       </c>
       <c r="D9" t="n">
-        <v>64.66</v>
+        <v>69.93000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JHANSI</t>
+          <t>CHANDAULI</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="C10" t="n">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="D10" t="n">
-        <v>63.67</v>
+        <v>69.31</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CHITRAKOOT</t>
+          <t>MAHARAJGANJ</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>134</v>
+        <v>320</v>
       </c>
       <c r="C11" t="n">
-        <v>85</v>
+        <v>219</v>
       </c>
       <c r="D11" t="n">
-        <v>63.43</v>
+        <v>68.44</v>
       </c>
     </row>
   </sheetData>
@@ -1936,129 +1936,129 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AZAMGARH</t>
+          <t>MAU</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>838</v>
+        <v>522</v>
       </c>
       <c r="C4" t="n">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="D4" t="n">
-        <v>11.69</v>
+        <v>15.71</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MAU</t>
+          <t>KUSHINAGAR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>522</v>
+        <v>413</v>
       </c>
       <c r="C5" t="n">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="D5" t="n">
-        <v>11.69</v>
+        <v>17.19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PRAYAGRAJ</t>
+          <t>MAINPURI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1181</v>
+        <v>516</v>
       </c>
       <c r="C6" t="n">
-        <v>183</v>
+        <v>89</v>
       </c>
       <c r="D6" t="n">
-        <v>15.5</v>
+        <v>17.25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AGRA</t>
+          <t>PRAYAGRAJ</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1077</v>
+        <v>1181</v>
       </c>
       <c r="C7" t="n">
-        <v>180</v>
+        <v>206</v>
       </c>
       <c r="D7" t="n">
-        <v>16.71</v>
+        <v>17.44</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>KUSHINAGAR</t>
+          <t>AZAMGARH</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>413</v>
+        <v>838</v>
       </c>
       <c r="C8" t="n">
-        <v>71</v>
+        <v>161</v>
       </c>
       <c r="D8" t="n">
-        <v>17.19</v>
+        <v>19.21</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MAINPURI</t>
+          <t>DEORIA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>516</v>
+        <v>580</v>
       </c>
       <c r="C9" t="n">
-        <v>89</v>
+        <v>113</v>
       </c>
       <c r="D9" t="n">
-        <v>17.25</v>
+        <v>19.48</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DEORIA</t>
+          <t>SANT KABIR NAGAR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>580</v>
+        <v>310</v>
       </c>
       <c r="C10" t="n">
-        <v>112</v>
+        <v>62</v>
       </c>
       <c r="D10" t="n">
-        <v>19.31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SANT KABIR NAGAR</t>
+          <t>SHAHJAHANPUR</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>310</v>
+        <v>430</v>
       </c>
       <c r="C11" t="n">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="D11" t="n">
-        <v>20</v>
+        <v>20.93</v>
       </c>
     </row>
   </sheetData>
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11687</v>
+        <v>13091</v>
       </c>
     </row>
     <row r="4">
@@ -2114,7 +2114,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>35.06</v>
+        <v>39.27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>